<commit_message>
Guía paso a paso de Alianza en Word y correcciones de la segunda revisión
- Nuevo alianza/Guia_Paso_a_Paso_Actualizacion_Plan_ALIANZA_DEL_ACERO.docx, generado desde el mismo contenido que la hoja PASO A PASO.
- Agrega puntos de atención, mapa completo diapositiva → celda del PPT, decisiones pendientes y anexo con el efecto de la fase B en la caja.
- Excel: textos corregidos en A1, A2, B3, B7, B8, C1, C4, D4, D5, E1, E3, E5, F1, F3, G2-G5, criterios 7 y 12, reglas de columnas y controles 13-15 y 23.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4oZnCzWT5uwD7Y9gLbehx
</commit_message>
<xml_diff>
--- a/alianza/Informe_Financiero_ALIANZA_DEL_ACERO_INFORME2_09062026_AJUSTADO_A_10_AÑOS_CON_GUIA.xlsx
+++ b/alianza/Informe_Financiero_ALIANZA_DEL_ACERO_INFORME2_09062026_AJUSTADO_A_10_AÑOS_CON_GUIA.xlsx
@@ -43502,7 +43502,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="339" t="inlineStr">
         <is>
-          <t>1. CONTROLES (todos deben quedar en OK antes de pasar al PowerPoint)</t>
+          <t>1. CONTROLES (todos en OK antes de pasar al PowerPoint, salvo el 13 si depende de la decisión de dividendos: ver paso E5)</t>
         </is>
       </c>
       <c r="C5" s="339"/>
@@ -44072,7 +44072,7 @@
       </c>
       <c r="H19" s="342" t="inlineStr">
         <is>
-          <t>E3: re-dimensionar los préstamos CP (Ej_Flujo fila 8) hasta que el saldo no sea negativo. Es normal que siga en REVISAR hasta terminar la fase E: la fase B lo empeora.</t>
+          <t>E3: redimensionar los préstamos CP (Ej_Flujo fila 8) hasta que el saldo no sea negativo. Es normal que siga en REVISAR hasta terminar la fase E: la fase B lo empeora.</t>
         </is>
       </c>
       <c r="I19" s="342"/>
@@ -44112,7 +44112,7 @@
       </c>
       <c r="H20" s="342" t="inlineStr">
         <is>
-          <t>E3: cada desembolso de la fila 8 necesita su devolución en la fila 16 antes de dic-2035.</t>
+          <t>E3: cada desembolso de la fila 8 necesita su devolución en la fila 16, a más tardar en dic-2035 (EA16).</t>
         </is>
       </c>
       <c r="I20" s="342"/>
@@ -44152,7 +44152,7 @@
       </c>
       <c r="H21" s="342" t="inlineStr">
         <is>
-          <t>E4: cablear Ej_Costos!R62:AC62 a Ej_Flujo fila 17 del mismo mes.</t>
+          <t>E4: vincular Ej_Costos!R62:AC62 a Ej_Flujo fila 17 del mismo mes.</t>
         </is>
       </c>
       <c r="I21" s="342"/>
@@ -44472,7 +44472,7 @@
       </c>
       <c r="H29" s="342" t="inlineStr">
         <is>
-          <t>E5: con utilidades menores a 500.000 (año 6) u 800.000 (año 7) el calendario fijo da negativo; consultar a la Dirección.</t>
+          <t>E5: con utilidades menores a 500.000 (año 6) u 800.000 (año 7) el calendario fijo da negativo; la Gerencia lo presenta a la Dirección.</t>
         </is>
       </c>
       <c r="I29" s="342"/>
@@ -46206,7 +46206,7 @@
     <row r="79" ht="20" customHeight="1">
       <c r="B79" s="339" t="inlineStr">
         <is>
-          <t>3. SERIES ANUALES PARA LOS GRÁFICOS (clic derecho en el gráfico &gt; Editar datos &gt; pegar la fila «Actualizado»)</t>
+          <t>3. SERIES ANUALES PARA LOS GRÁFICOS (copiar E:N de la fila «Actualizado»; en el PPT: Editar datos &gt; primera celda de la serie &gt; Pegado especial &gt; Valores + Transponer; ver paso G1)</t>
         </is>
       </c>
       <c r="C79" s="339"/>
@@ -47972,7 +47972,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="B3" s="363" t="inlineStr">
         <is>
-          <t>Alianza del Acero · Modelo a 10 años (Año 1 = 2026 … Año 10 = 2035) · Libro base: INFORME2 ajustado a 10 años (09/06/2026) · Guía preparada el 13/10/2026 · Controles y datos para el PowerPoint en la hoja «CONTROLES Y PPT».</t>
+          <t>Alianza del Acero · Modelo a 10 años (Año 1 = 2026 … Año 10 = 2035) · Libro base: INFORME2 ajustado a 10 años (09/06/2026) · Guía preparada el 13/10/2026 y actualizada el 16/10/2026 · Controles y datos para el PowerPoint en la hoja «CONTROLES Y PPT».</t>
         </is>
       </c>
       <c r="C3" s="363"/>
@@ -47999,7 +47999,7 @@
       </c>
       <c r="C6" s="367" t="inlineStr">
         <is>
-          <t>Seguir las fases en orden: A Preparar → B Correcciones únicas → C Ventas → D Costos → E Caja y préstamos CP → F Resultados y controles → G PowerPoint. Al terminar cada fase presionar F9 y revisar en «CONTROLES Y PPT» los controles que indica cada paso (columna «Control / resultado esperado»). Los controles 13, 14 y 23 (caja, préstamos CP y dividendos) recién deben quedar en OK al terminar la fase E; en el paso F1, todos.</t>
+          <t>Seguir las fases en orden: A Preparar → B Correcciones únicas → C Ventas → D Costos → E Caja y préstamos CP → F Resultados y controles → G PowerPoint. Al terminar cada fase presionar F9 y revisar en «CONTROLES Y PPT» los controles que indica cada paso (columna «Control / resultado esperado»). Los controles 13, 14 y 23 (caja, préstamos CP y dividendos) recién deben quedar en OK al terminar la fase E; en el paso F1, todos (salvo el 13 si depende de la decisión de dividendos: paso E5).</t>
         </is>
       </c>
       <c r="D6" s="367"/>
@@ -48051,7 +48051,7 @@
       <c r="E9" s="367"/>
       <c r="F9" s="367"/>
     </row>
-    <row r="10" ht="43.6" customHeight="1">
+    <row r="10" ht="56.8" customHeight="1">
       <c r="B10" s="369" t="inlineStr">
         <is>
           <t>•</t>
@@ -48059,7 +48059,7 @@
       </c>
       <c r="C10" s="367" t="inlineStr">
         <is>
-          <t>Escribir solo en las celdas indicadas. No escribir en columnas de total o promedio (O y AD de las hojas Ej_; O, AB, AO, BB, BO, CB, CO, DB, DO, EB y EF de Ej_Flujo), salvo las celdas que un paso indica expresamente: Ej_Producción!O31:O32 y O46:O47 (B4), Ej_Costos!O9:O19 y AD9:AD19 (B5), Ej_Costos!O1 (D2) y Ej_Flujo!O37 y O40 (E2). Tampoco en el plan original (columnas P y AE de las hojas Ej_; columna E de Supuestos).</t>
+          <t>Escribir solo en las celdas indicadas. No escribir en columnas de total o promedio (O y AD de Ej_Producción, Ej_Ingresos, Ej_Costos, Ej_Resultados y Ej_Deuda; O, AB, AO, BB, BO, CB, CO, DB, DO, EB y EF de Ej_Flujo), salvo las celdas que un paso indica expresamente: Ej_Producción!O31:O32 y O46:O47 (B4), Ej_Costos!O9:O19 y AD9:AD19 (B5), Ej_Costos!O1 (D2) y Ej_Flujo!O37 y O40 (E2). Tampoco en el plan original (columnas P y AE de esas cinco hojas; columna E de Supuestos). En Ej_Flujo no hay columnas de plan: P, AD y AE son meses (ene-2027, feb-2028 y mar-2028) y se editan cuando un paso lo indica. El auxiliar Ej_Costos!O88:P114 (paso D5) no es plan ni total.</t>
         </is>
       </c>
       <c r="D10" s="367"/>
@@ -48224,7 +48224,7 @@
       </c>
       <c r="D21" s="367" t="inlineStr">
         <is>
-          <t>Días de Supuestos!B77:B83: caja 2, sueldos 15, stock MP 45, ventas a crédito 90, proveedores menores 15. En el flujo mensual, las ventas se cobran a los 3 meses.</t>
+          <t>Días de Supuestos!B77:B83: caja 2, sueldos 15, stock MP 45, ventas a crédito 90, producto terminado 0, crédito de proveedores de MP 0 (sin crédito del proveedor de chapa) y proveedores menores 15. En el flujo mensual, las ventas se cobran a los 3 meses.</t>
         </is>
       </c>
       <c r="E21" s="367"/>
@@ -48298,7 +48298,7 @@
       <c r="E25" s="367"/>
       <c r="F25" s="367"/>
     </row>
-    <row r="26" ht="30.4" customHeight="1">
+    <row r="26" ht="43.6" customHeight="1">
       <c r="B26" s="369">
         <v>12</v>
       </c>
@@ -48309,7 +48309,7 @@
       </c>
       <c r="D26" s="367" t="inlineStr">
         <is>
-          <t>En el libro solo están el plan de los años 1 y 2 (columnas P y AE de las hojas Ej_) y los supuestos originales (Supuestos, columna E). El VAN y la TIR del plan y las series de los años 3-10 están en «CONTROLES Y PPT», sección 4.</t>
+          <t>En el libro solo están el plan de los años 1 y 2 (columnas P y AE de Ej_Producción, Ej_Ingresos, Ej_Costos, Ej_Resultados y Ej_Deuda) y los supuestos originales (Supuestos, columna E). En «CONTROLES Y PPT», el VAN, la TIR, el payback y los rótulos acumulados del plan están en la sección 4, y las series plan de los gráficos (los 10 años, copiadas del PPT de junio) en la sección 3, filas 82, 85, 87 y 89.</t>
         </is>
       </c>
       <c r="E26" s="367"/>
@@ -48353,7 +48353,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="30.4" customHeight="1">
+    <row r="30" ht="70.0" customHeight="1">
       <c r="B30" s="370" t="inlineStr">
         <is>
           <t>A1</t>
@@ -48371,16 +48371,16 @@
       </c>
       <c r="E30" s="367" t="inlineStr">
         <is>
-          <t>Archivo &gt; Guardar como: «…_RV01_PROSPECCION_AAAAMMDD.xlsx». Trabajar siempre sobre la copia y conservar la versión anterior para comparar.</t>
+          <t>Archivo &gt; Guardar como: «…_RV01_PROSPECCION_AAAAMMDD.xlsx». Trabajar siempre sobre la copia y conservar la versión anterior para comparar. Antes de la fase G, hacer lo mismo con el PowerPoint (Informe_Ejecutivo_Plan_vs_Actualizado_ALIANZA_DEL_ACERO_10_AÑOS.pptx): guardarlo con un nombre nuevo («…_RV01_AAAAMMDD.pptx») y editar solo la copia.</t>
         </is>
       </c>
       <c r="F30" s="367" t="inlineStr">
         <is>
-          <t>El nombre del archivo indica versión y fecha.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="43.6" customHeight="1">
+          <t>Los nombres del libro y del PPT indican versión y fecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="56.8" customHeight="1">
       <c r="B31" s="370" t="inlineStr">
         <is>
           <t>A2</t>
@@ -48398,12 +48398,12 @@
       </c>
       <c r="E31" s="367" t="inlineStr">
         <is>
-          <t>Datos &gt; Editar vínculos. Ante el aviso de vínculos externos, elegir «No actualizar»: la deuda LP de 'Servicio Deuda'!D18:I20 viene del archivo CALCULADORA PRESTAMO, que no está en este equipo. Fórmulas &gt; Opciones para el cálculo &gt; Automático.</t>
+          <t>Al abrir el libro, ante el aviso de vínculos externos, elegir «No actualizar»: la deuda LP de 'Servicio Deuda'!D18:I20 viene del archivo CALCULADORA PRESTAMO, que no está en este equipo. En Datos &gt; Editar vínculos se puede confirmar que el vínculo quedó sin actualizar. Fórmulas &gt; Opciones para el cálculo &gt; Automático.</t>
         </is>
       </c>
       <c r="F31" s="367" t="inlineStr">
         <is>
-          <t>'Servicio Deuda'!D18 sigue en 29.277,76, sin error.</t>
+          <t>Después del paso A3 (la hoja Servicio Deuda está oculta): 'Servicio Deuda'!D18 sigue en 29.277,76, sin error.</t>
         </is>
       </c>
     </row>
@@ -48598,7 +48598,7 @@
       </c>
       <c r="E40" s="367" t="inlineStr">
         <is>
-          <t>Opción exacta: AC23:AN23 =('Servicio Deuda'!$F$23+'Servicio Deuda'!$F$24+'Servicio Deuda'!$F$25)/12; AP23:BA23 igual con la columna G; BC23:BN23 con la H; BP23:BY23 =('Servicio Deuda'!$I$23+'Servicio Deuda'!$I$24+'Servicio Deuda'!$I$25)/10. Agrega unos USD 464.000 de egresos en jul-oct 2031 (4 × 116.058) y, neto de la baja de las cuotas 2028-2030, unos USD 387.000 (= valor actual del control 17). Después hay que revisar los préstamos CP (paso E3).</t>
+          <t>AC23:AN23 =('Servicio Deuda'!$F$23+'Servicio Deuda'!$F$24+'Servicio Deuda'!$F$25)/12; AP23:BA23 igual con la columna G; BC23:BN23 con la H; BP23:BY23 =('Servicio Deuda'!$I$23+'Servicio Deuda'!$I$24+'Servicio Deuda'!$I$25)/10. Agrega unos USD 464.000 de egresos en jul-oct 2031 (4 × 116.058) y, neto de la baja de las cuotas de ene-2028 a jun-2031 (≈ USD 77.000), unos USD 387.000 (≈ valor actual del control 17). Después hay que revisar los préstamos CP (paso E3).</t>
         </is>
       </c>
       <c r="F40" s="367" t="inlineStr">
@@ -48688,7 +48688,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="70.0" customHeight="1">
+    <row r="44" ht="96.4" customHeight="1">
       <c r="B44" s="370" t="inlineStr">
         <is>
           <t>B7</t>
@@ -48706,7 +48706,7 @@
       </c>
       <c r="E44" s="367" t="inlineStr">
         <is>
-          <t>B8 «Payback inversión propia (años)». C8 =SI.ERROR(CONTAR.SI(D7:M7;"&lt;0")+(-INDICE(C7:M7;CONTAR.SI(C7:M7;"&lt;0")))/INDICE(C6:M6;CONTAR.SI(C7:M7;"&lt;0")+1);"No recupera en 10 años"). B13 «Payback inversión total (años)» y en C13 la misma fórmula sobre las filas 11 (flujo) y 12 (acumulado). Luego Dashboard!C12 =Payback!C8 y C13 =Payback!C13, con formato 0,0 "años".</t>
+          <t>En Payback!B8 escribir el rótulo «Payback inversión propia (años)» y en Payback!C8: =SI.ERROR(CONTAR.SI(D7:M7;"&lt;0")+(-INDICE(C7:M7;CONTAR.SI(C7:M7;"&lt;0")))/INDICE(C6:M6;CONTAR.SI(C7:M7;"&lt;0")+1);"No recupera en 10 años"). En Payback!B13 escribir «Payback inversión total (años)» y en Payback!C13: =SI.ERROR(CONTAR.SI(D12:M12;"&lt;0")+(-INDICE(C12:M12;CONTAR.SI(C12:M12;"&lt;0")))/INDICE(C11:M11;CONTAR.SI(C12:M12;"&lt;0")+1);"No recupera en 10 años"). Luego Dashboard!C12 =Payback!C8 y Dashboard!C13 =Payback!C13 (hoy dicen «4 Años» y «7 Años» tipeados), con formato 0,0 "años".</t>
         </is>
       </c>
       <c r="F44" s="367" t="inlineStr">
@@ -48715,7 +48715,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="188.8" customHeight="1">
+    <row r="45" ht="202.0" customHeight="1">
       <c r="B45" s="370" t="inlineStr">
         <is>
           <t>B8</t>
@@ -48733,7 +48733,7 @@
       </c>
       <c r="E45" s="367" t="inlineStr">
         <is>
-          <t>Mismo mapeo que 2027, con el costo anual de la hoja Costos / 12. Para 2028: AC13:AN13 =(Costos!$F$10+Costos!$F$13+Costos!$F$27)/12 (insumos, packaging y honorarios); AC19:AN19 =(Costos!$F$7+Costos!$F$8+Costos!$F$14+Costos!$F$20+Costos!$F$21)/12 (nómina y alimentación); AC21:AN21 =(Costos!$F$16+Costos!$F$22+Costos!$F$23)/12 (energía, servicios y alquileres); AC22:AN22 =(Costos!$F$9+Costos!$F$11+Costos!$F$12+Costos!$F$15+Costos!$F$24+Costos!$F$25+Costos!$F$26)/12 (otros). Repetir con la columna G de Costos en AP:BA, H en BC:BN, I en BP:CA, J en CC:CN, K en CP:DA, L en DC:DN y M en DP:EA, sin escribir en las columnas de total. Hoy esas filas repiten los montos de 2027 y no siguen al volumen: el cambio agrega ≈ USD 1,62M de egresos en 2028-2035. Atención: la fila 25 («Inversiones / CAPEX») repite desde feb-2027 los servicios de terceros de Steel Frame que ya están en la fila 22 (USD 3.750/mes; 371.250 en 2027-2035). Confirmarlo con quien armó el modelo; si es una duplicación, dejar en 0 las columnas de mes de la fila 25 desde feb-2027 y anotarlo en el registro.</t>
+          <t>Mismo mapeo que 2027, con el costo anual de la hoja Costos / 12. Para 2028: AC13:AN13 =(Costos!$F$10+Costos!$F$13+Costos!$F$27)/12 (insumos, packaging y honorarios); AC19:AN19 =(Costos!$F$7+Costos!$F$8+Costos!$F$14+Costos!$F$20+Costos!$F$21)/12 (nómina y alimentación); AC21:AN21 =(Costos!$F$16+Costos!$F$22+Costos!$F$23)/12 (energía, servicios y alquileres); AC22:AN22 =(Costos!$F$9+Costos!$F$11+Costos!$F$12+Costos!$F$15+Costos!$F$24+Costos!$F$25+Costos!$F$26)/12 (otros). Repetir con la columna G de Costos en AP:BA, H en BC:BN, I en BP:CA, J en CC:CN, K en CP:DA, L en DC:DN y M en DP:EA, sin escribir en las columnas de total. Hoy esas filas son valores pegados, iguales en los ocho años 2028-2035 (parecidos a 2027, pero no iguales en las filas 13 y 22), y no siguen al volumen: el cambio agrega ≈ USD 1,62M de egresos en 2028-2035. Atención: la fila 25 («Inversiones / CAPEX») repite desde feb-2027 los servicios de terceros de Steel Frame que ya están en la fila 22 (USD 3.750/mes; 371.250 en 2027-2035). Confirmarlo con quien armó el modelo; si es una duplicación, dejar en 0 las columnas de mes de la fila 25 desde feb-2027 y anotarlo en el registro.</t>
         </is>
       </c>
       <c r="F45" s="367" t="inlineStr">
@@ -48780,7 +48780,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="109.6" customHeight="1">
+    <row r="49" ht="136.0" customHeight="1">
       <c r="B49" s="370" t="inlineStr">
         <is>
           <t>C1</t>
@@ -48798,7 +48798,7 @@
       </c>
       <c r="E49" s="367" t="inlineStr">
         <is>
-          <t>Rangos: Ej_Producción!H22:K32 (producción) y H37:K47 (ventas); Ej_Ingresos!G8:K18 (precio). Desde el primer mes no real hasta el corte (hoy: volumen desde junio, columna H; precio desde mayo, columna G). Producción en Tn producidas y ventas en Tn facturadas, por producto y mes. Precio = facturación del mes en USD sin IVA ÷ Tn vendidas del mismo producto (si se facturó en Gs, convertir con el TC del mes). Mes sin venta: Tn = 0. Pasar los meses reales a formato azul (Copiar formato desde C22 y C8) y actualizar los títulos B2 («…EJECUTADO A &lt;MES&gt;…») de Ej_Producción, Ej_Ingresos y Ej_Costos.</t>
+          <t>Rangos (ejemplo con corte a setiembre; si el corte es otro, terminar en la columna de ese mes): Ej_Producción!H22:K32 (producción) y H37:K47 (ventas); Ej_Ingresos!G8:K18 (precio). Desde el primer mes no real (hoy: volumen desde junio, columna H; precio desde mayo, columna G) hasta el mes del corte (setiembre = columna K). Producción en Tn producidas y ventas en Tn facturadas, por producto y mes. Precio = facturación del mes en USD sin IVA ÷ Tn vendidas del mismo producto (si se facturó en Gs, convertir con el TC del mes). Mes sin venta: Tn = 0. Pasar los meses reales a formato azul (Copiar formato desde C22 y C8) y actualizar los títulos B2: en Ej_Producción y Ej_Ingresos, «…EJECUTADO A ABRIL…» → mes del corte; en Ej_Costos, «…EJECUTADO &amp; PROYECTADO» → «…EJECUTADO A &lt;MES&gt; &amp; PROYECTADO».</t>
         </is>
       </c>
       <c r="F49" s="367" t="inlineStr">
@@ -48884,7 +48884,7 @@
       </c>
       <c r="F52" s="367" t="inlineStr">
         <is>
-          <t>Producción!F6/E6 − 1 = B11 en cada producto.</t>
+          <t>Producción!F6/E6 − 1 ≈ B11 en cada producto (por el redondeo a Tn enteras difiere hasta ±0,2 puntos; hoy da entre 4,96% y 5,15% con B11 = 5%).</t>
         </is>
       </c>
     </row>
@@ -49115,7 +49115,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="56.8" customHeight="1">
+    <row r="63" ht="70.0" customHeight="1">
       <c r="B63" s="370" t="inlineStr">
         <is>
           <t>D4</t>
@@ -49133,7 +49133,7 @@
       </c>
       <c r="E63" s="367" t="inlineStr">
         <is>
-          <t>Rango: G34:K54 (meses cerrados). Mismo criterio que ene-abr: los montos en Gs se cargan como =MontoGs/USD (p. ej. =29898626/USD), encima de la fórmula de proyección del mes. Los meses sin gasto, en 0. Las filas 35 y 48 quedan en 0 porque las cargas sociales ya están en las filas 34 y 47.</t>
+          <t>Rango (ejemplo con corte a setiembre): G34:K54 (may-sep, meses cerrados). Mismo criterio que ene-abr: los montos en Gs se cargan como =MontoGs/USD (p. ej. =29898626/USD), encima de la fórmula de proyección del mes. Los meses sin gasto, en 0. Las filas 35 y 48 quedan en 0 porque las cargas sociales ya están en las filas 34 y 47.</t>
         </is>
       </c>
       <c r="F63" s="367" t="inlineStr">
@@ -49165,7 +49165,7 @@
       </c>
       <c r="F64" s="367" t="inlineStr">
         <is>
-          <t>MO año 2 → año 3 crece ≈ 3,8%.</t>
+          <t>=(Costos!F7+Costos!F8+Costos!F20+Costos!F21)/(Costos!E7+Costos!E8+Costos!E20+Costos!E21)-1 ≈ 3,8% (= 1,03 × 1,4309 / 1,42 − 1, cualquiera sea la dotación de 2027).</t>
         </is>
       </c>
     </row>
@@ -49288,7 +49288,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="43.6" customHeight="1">
+    <row r="71" ht="96.4" customHeight="1">
       <c r="B71" s="370" t="inlineStr">
         <is>
           <t>E1</t>
@@ -49306,7 +49306,7 @@
       </c>
       <c r="E71" s="367" t="inlineStr">
         <is>
-          <t>Mantener 2 / 15 / 45 / 90 / 0 / 0 / 15 salvo un cambio de política. Si cambia B80 (cobro), también hay que mover el desfase de los cobros de Ej_Flujo fila 6 (hoy fijo en 3 meses) y corregir los rótulos de Capital Trabajo!B7:B15.</t>
+          <t>Mantener B77 caja 2, B78 sueldos 15, B79 stock MP 45, B80 ventas a crédito 90, B81 producto terminado 0, B82 crédito de proveedores de MP 0 y B83 proveedores menores 15 (días), salvo un cambio de política. Si cambia B80 (cobro), también hay que mover el desfase de los cobros de Ej_Flujo fila 6 (hoy cada mes cobra la venta de 3 meses antes; p. ej. F6 =+Ej_Ingresos!C34 cobra en abril la venta de enero) y corregir los rótulos de Capital Trabajo!B7:B15. Ese desfase solo afecta la caja mensual: el VAN toma el capital de trabajo de la hoja Capital Trabajo.</t>
         </is>
       </c>
       <c r="F71" s="367" t="inlineStr">
@@ -49342,7 +49342,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="188.8" customHeight="1">
+    <row r="73" ht="202.0" customHeight="1">
       <c r="B73" s="370" t="inlineStr">
         <is>
           <t>E3</t>
@@ -49350,7 +49350,7 @@
       </c>
       <c r="C73" s="368" t="inlineStr">
         <is>
-          <t>Re-dimensionar los préstamos CP para chapas</t>
+          <t>Redimensionar los préstamos CP para chapas</t>
         </is>
       </c>
       <c r="D73" s="371" t="inlineStr">
@@ -49360,12 +49360,12 @@
       </c>
       <c r="E73" s="367" t="inlineStr">
         <is>
-          <t>Filas 8, 16, 17 y 29 (solo columnas de mes). Con B1-B3 y la prospección cargados, recorrer el saldo mensual (fila 29) desde ago-2026. Para cada préstamo: (a) monto en la fila 8 del mes de desembolso (múltiplos de 100.000); (b) en la fila 16 del mes de devolución =+&lt;celda de la fila 8&gt; (ej. V16 =+P8); (c) en la fila 17 de esa columna =((8%/365)*DÍAS)*&lt;celda fila 16&gt;, con DÍAS = 30 × meses (ene→jul = 180); (d) si se mueve o elimina un desembolso, mover o borrar también su devolución y su interés; (e) un préstamo CP en 2026 se carga igual; si se devuelve dentro de 2026, sumar su interés en Ej_Costos (paso E4). L16 (2.779.626) y L17 (125.862) son la devolución a CIE S.A., no préstamos CP: no tocarlas. Meta: saldo ≥ 0 todos los meses, con un colchón de 100.000 a 400.000, y todo devuelto antes de dic-2035. Antes de la fase B el único déficit es ago-2032 (CJ29 = −245.726). Después de la fase B, con los datos actuales, hay faltantes de calce desde abr-2030 (máximo −736.000 en ago-2032 sin contar dividendos) y el saldo de dic-2035 queda en ≈ −2,22M después de los dividendos: ver E5.</t>
+          <t>Se escribe en las filas 8, 16 y 17 (solo columnas de mes); la fila 29 (saldo acumulado) es fórmula y solo se lee. Con la fase B completa (B1-B8) y la prospección cargada, recorrer el saldo mensual (fila 29) desde ago-2026. Para cada préstamo: (a) monto en la fila 8 del mes de desembolso (múltiplos de 100.000); (b) en la fila 16 del mes de devolución =+&lt;celda de la fila 8&gt; (ej. V16 =+P8); (c) en la fila 17 de esa columna =((8%/365)*DÍAS)*&lt;celda fila 16&gt;, con DÍAS = 30 × meses (ene→jul = 180); (d) si se mueve o elimina un desembolso, mover o borrar también su devolución y su interés; (e) un préstamo CP en 2026 se carga igual; si se devuelve dentro de 2026, sumar su interés en Ej_Costos (paso E4). L16 (2.779.626) y L17 (125.862) son la devolución a CIE S.A., no préstamos CP: no tocarlas. Meta: saldo ≥ 0 todos los meses, con un colchón de 100.000 a 400.000, y todo devuelto a más tardar en dic-2035 (columna EA). Antes de la fase B el único déficit es ago-2032 (CJ29 = −245.726). Después de la fase B, con los datos actuales, hay faltantes de calce desde abr-2030 (máximo −736.000 en ago-2032 sin contar dividendos) y el saldo de dic-2035 queda en ≈ −2,22M después de los dividendos: ver E5.</t>
         </is>
       </c>
       <c r="F73" s="367" t="inlineStr">
         <is>
-          <t>Controles 13 y 14 en OK.</t>
+          <t>Controles 13 y 14 en OK (el 13, salvo que dependa de la decisión de dividendos: paso E5).</t>
         </is>
       </c>
     </row>
@@ -49396,7 +49396,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="122.8" customHeight="1">
+    <row r="75" ht="175.6" customHeight="1">
       <c r="B75" s="370" t="inlineStr">
         <is>
           <t>E5</t>
@@ -49414,7 +49414,7 @@
       </c>
       <c r="E75" s="367" t="inlineStr">
         <is>
-          <t>Las nuevas utilidades cambian los dividendos (Resultados fila 18; calendario fijo desde 2031, con montos tipeados de 500.000 y 800.000), que se pagan en diciembre en Ej_Flujo fila 20 (CA20, CN20, DA20, DN20 y EA20; esa fila no tiene totales anuales). Si cambia la caja, volver a E3 hasta que el saldo mínimo se estabilice (2 o 3 vueltas). Si con todos los CP devueltos el saldo de dic-2035 sigue negativo (hoy ≈ −2,22M después de la fase B, con ≈ USD 10M de dividendos en 2031-2035), el calendario de dividendos excede la caja disponible: presentar a la Gerencia las alternativas (diferir o reducir dividendos, mantener deuda CP al cierre o refinanciar a largo plazo). No cambiar la política sin instrucción de la Dirección.</t>
+          <t>Las nuevas utilidades cambian los dividendos (Resultados fila 18, calculados en las filas 25-31 sobre la retención de utilidades de la fila 17). El calendario es fijo: en 2031 se paga el 50% de la utilidad de 2027; en 2032, el otro 50% de 2027 y la de 2028; en 2033, la de 2029; en 2034, la de 2030 y 500.000 de la de 2031 (H29, tipeado); en 2035, el resto de 2031 y 800.000 de la de 2032 (I30, tipeado). Se pagan en diciembre en Ej_Flujo fila 20 (CA20, CN20, DA20, DN20 y EA20; esa fila no tiene totales anuales). Si cambia la caja, volver a E3 hasta que el saldo mínimo se estabilice (2 o 3 vueltas). Si con todos los CP devueltos el saldo de dic-2035 sigue negativo (hoy ≈ −2,22M después de la fase B, con ≈ USD 10M de dividendos en 2031-2035), el calendario de dividendos excede la caja disponible: la Gerencia presenta a la Dirección las alternativas (diferir o reducir dividendos, mantener deuda CP al cierre o refinanciar a largo plazo). No cambiar la política sin instrucción de la Dirección.</t>
         </is>
       </c>
       <c r="F75" s="367" t="inlineStr">
@@ -49461,7 +49461,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="56.8" customHeight="1">
+    <row r="79" ht="122.8" customHeight="1">
       <c r="B79" s="370" t="inlineStr">
         <is>
           <t>F1</t>
@@ -49479,12 +49479,12 @@
       </c>
       <c r="E79" s="367" t="inlineStr">
         <is>
-          <t>Presionar F9 (o Ctrl+Alt+F9). Todos los controles deben quedar en OK; la última columna indica qué paso revisar. Con el libro tal como llegó hay 8 controles en REVISAR: el 9, 11, 12, 17, 21, 22 y 26 se corrigen en la fase B; el 13 (déficit de caja) se corrige en E3 y E5, y empeora después de la fase B.</t>
+          <t>Presionar F9 (o Ctrl+Alt+F9). Todos los controles deben quedar en OK; la última columna indica qué paso revisar. Con el libro tal como llegó hay 8 controles en REVISAR: el 9, 11, 12, 17, 21, 22 y 26 se corrigen en la fase B; el 13 (déficit de caja) se corrige en E3 y E5, y empeora después de la fase B. Excepción: si el control 13 solo puede pasar a OK cambiando la política de dividendos o dejando préstamos CP sin devolver al cierre (control 14), no forzarlo: dejarlo en REVISAR, anotar en el registro el saldo de dic-2035 y las alternativas presentadas (paso E5) y seguir con la fase G, aclarando en el PPT que la caja 2031-2035 depende de esa decisión.</t>
         </is>
       </c>
       <c r="F79" s="367" t="inlineStr">
         <is>
-          <t>26 de 26 controles en OK.</t>
+          <t>26 de 26 controles en OK, o 25 de 26 con el control 13 pendiente de la decisión de dividendos y anotado en el registro.</t>
         </is>
       </c>
     </row>
@@ -49526,9 +49526,9 @@
           <t>Registrar la actualización</t>
         </is>
       </c>
-      <c r="D81" s="367" t="inlineStr">
-        <is>
-          <t>Registro al final de esta hoja</t>
+      <c r="D81" s="371" t="inlineStr">
+        <is>
+          <t>Registro de actualizaciones</t>
         </is>
       </c>
       <c r="E81" s="367" t="inlineStr">
@@ -49607,7 +49607,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="70.0" customHeight="1">
+    <row r="86" ht="83.2" customHeight="1">
       <c r="B86" s="370" t="inlineStr">
         <is>
           <t>G2</t>
@@ -49625,7 +49625,7 @@
       </c>
       <c r="E86" s="367" t="inlineStr">
         <is>
-          <t>Copiar cada valor de la columna «Libro (vivo)» con el redondeo de la diapositiva (USD con separador de miles; % con 1 decimal; diferencias de TIR en puntos porcentuales). Las variaciones contra el plan se calculan contra los rótulos plan del PPT (sección 4: 150K Tn, USD 180M, USD 21,1M y USD 17,8M), con el mismo criterio que la versión de junio; así la tabla de la diap. 3 queda coherente.</t>
+          <t>Copiar cada valor de la columna «Libro (vivo)» con el redondeo de la diapositiva (USD con separador de miles; % con 1 decimal; diferencias de TIR en puntos porcentuales). Las variaciones contra el plan se calculan contra los rótulos plan del PPT (sección 4 de «CONTROLES Y PPT»: 150K Tn, USD 180M, USD 21,1M y USD 17,8M), con el mismo criterio que la versión de junio; así la tabla de la diap. 3 queda coherente.</t>
         </is>
       </c>
       <c r="F86" s="367" t="inlineStr">
@@ -49634,7 +49634,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="136.0" customHeight="1">
+    <row r="87" ht="320.8" customHeight="1">
       <c r="B87" s="370" t="inlineStr">
         <is>
           <t>G3</t>
@@ -49652,16 +49652,16 @@
       </c>
       <c r="E87" s="367" t="inlineStr">
         <is>
-          <t>Buscar (Ctrl+F) cada cifra que cambió y reemplazarla en todas las diapositivas donde se repite. Corregir además los errores de la versión de junio: acumulados de ingresos (217M → 215,6M), EBITDA (26,4M → 25,4M) y utilidad neta (19,6M → 18,0M); variaciones +21% / +25% / +10% / +7%; TIR −0,29 → −0,27 pp; margen de seguridad 52-69% → 50-69%; préstamos CP 5-12M → 4-12M; «11 productos activos en el año 1» (son 9); materia prima acumulada 183M → 181,1M (diap. 6); desvío del costo de MP 6-16% → 2,7-15,8%, o «5,9-15,8% sin Accesorios» si se documenta (diap. 2, 6, 11 y 13); en la diap. 13, «USD 4-7M adicionales» = indicadores 31 y 32. El 95,3% de MP/costos del plan (diap. 6) es un valor plan: no cambiarlo sin definir la fuente oficial del plan (sección 4). Rotular el año 1 como «real a &lt;mes&gt; + proyección».</t>
+          <t>Buscar (Ctrl+F) cada cifra que cambió y reemplazarla en todas las diapositivas donde se repite, siempre con el valor vivo de las secciones 2 y 3 de «CONTROLES Y PPT» (con el libro ya actualizado). La versión de junio, además, tenía cifras que no coincidían con el libro de ese momento; como referencia (PPT de junio → libro de junio): ingresos acumulados 217M → 215,6M; EBITDA acumulado 26,4M → 25,4M; utilidad neta acumulada 19,6M → 18,0M; variaciones contra el plan +7% → +7,5% (producción, indicador 13; diap. 3, 4 y 13), +21% → +19,8% (ingresos, indicador 15; diap. 3, 5, 9 y 13), +25% → +20,4% (EBITDA, indicador 17; diap. 3, 7, 9 y 13) y +10% → +1,3% (utilidad neta, indicador 19; diap. 3); el «+25%» de la diap. 5 es otro dato (ingresos del año 10 contra el plan, hoy +25,3%): no reemplazarlo por el del EBITDA; TIR −0,29 → −0,27 pp; margen de seguridad 52-69% → 50-69% (diap. 10); préstamos CP «5-12M» → «4-12M» (diap. 11 y 13) y «5-11.9M» → «4-11.9M» (diap. 8); «11 vs 8 productos activos en Año 1» → «9 vs 8» (diap. 4); materia prima acumulada 183M → 181,1M (diap. 6); desvío del costo de MP 6-16% → 2,7-15,8%, o «5,9-15,8% sin Accesorios» si se documenta (diap. 2, 6, 11 y 13). Revisar también dos frases que no coinciden con las series: diap. 7, «los márgenes EBITDA actualizados son superiores en años 2-5» (solo el año 2 supera al plan: 14,1% frente a 12,8%; el año 3 queda igual y los años 4 a 10, por debajo); diap. 10, «a partir del Año 6 (fin de deuda LP), el PE baja significativamente» (sube de 6.204 Tn en el año 5 a 6.433 en el año 6, baja a 5.492 en el año 7 y vuelve a subir hasta 7.854 en el año 10). En la diap. 13, «USD 4-7M adicionales» = indicadores 31 y 32. El 95,3% de MP/costos del plan (diap. 6) es un valor plan: no cambiarlo sin definir la fuente oficial del plan (sección 4 de «CONTROLES Y PPT»). Rotular el año 1 como «real a &lt;mes&gt; + proyección».</t>
         </is>
       </c>
       <c r="F87" s="367" t="inlineStr">
         <is>
-          <t>Cada cifra del PPT = celda de la sección 2 o 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="43.6" customHeight="1">
+          <t>Cada cifra del PPT = celda de la sección 2 o 3 de «CONTROLES Y PPT».</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="96.4" customHeight="1">
       <c r="B88" s="370" t="inlineStr">
         <is>
           <t>G4</t>
@@ -49679,7 +49679,7 @@
       </c>
       <c r="E88" s="367" t="inlineStr">
         <is>
-          <t>Usar el valor calculado de la sección 2 (inversión propia 6,4 años: se recupera durante el año 7), no el texto del Dashboard. Indicar el criterio: dividendos descontados a Ke.</t>
+          <t>Usar el valor calculado de la sección 2 de «CONTROLES Y PPT» (indicador 38: hoy 6,4 años; se recupera durante el año 7), no el texto del Dashboard. Actualizar también la diferencia contra el plan («(+3)»; plan = 3 años, sección 4 de «CONTROLES Y PPT») y la frase de la conclusión «extienden el Payback de inversión propia en 3 años más». En la nota «El Payback es considerado desde el año 6…», indicar el criterio del modelo: dividendos descontados a Ke (16,32%) contra el aporte propio (USD 606.000), con dividendos desde 2031 (año 6).</t>
         </is>
       </c>
       <c r="F88" s="367" t="inlineStr">
@@ -49688,7 +49688,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="162.4" customHeight="1">
+    <row r="89" ht="228.4" customHeight="1">
       <c r="B89" s="370" t="inlineStr">
         <is>
           <t>G5</t>
@@ -49706,7 +49706,7 @@
       </c>
       <c r="E89" s="367" t="inlineStr">
         <is>
-          <t>El libro no tiene cálculo de sensibilidad. Para cada variable, en una COPIA: aplicar el cambio (precio: Ej_Ingresos!L8:N18 y R8:AC18 × 1,05; costo de MP: Ej_Costos!L9:N19 y R9:AC19 × 1,05; volumen: Ej_Producción L22:N32, L37:N47, R22:AC32 y R37:AC47 × 1,10; cobranza: Supuestos!B80 = 60 y desfase de 2 meses en Ej_Flujo fila 6), anotar VAN-TIR!C24 y restar el VAN base. Atención: una réplica del modelo da ≈ ±USD 5,9M de VAN por ±5% de precio y ≈ ∓USD 5,2M por ±5% de MP, muy por encima de lo que muestra la diapositiva de junio (±1,2M y ±1,0M). Tasa CP +2% y tipo de cambio ±10%: con este libro el VAN no cambia (el interés CP no entra al VAN y las proyecciones están en USD); informar ≈ 0 en VAN y, si se quiere mostrar, el efecto en la utilidad neta acumulada y en la caja (la tasa CP exige cambiar el 8% de cada fórmula de Ej_Flujo fila 17). Aplicar los cambios a todos los meses posteriores al corte (con corte a setiembre, L:N).</t>
+          <t>El libro no tiene cálculo de sensibilidad. Para cada variable, en una COPIA del libro ya actualizado, aplicar el cambio a todos los meses posteriores al corte (con corte a setiembre: L:N de 2026 y R:AC de 2027; los años 3-10 se ajustan solos porque parten de 2027; si se usaron Prosp_Tn o Prosp_Precio, aplicar el mismo factor en esas hojas): precio, Ej_Ingresos!L8:N18 y R8:AC18 × 1,05; costo de MP, Ej_Costos!L9:N19 y R9:AC19 × 1,05; volumen, Ej_Producción!L22:N32, L37:N47, R22:AC32 y R37:AC47 × 1,10; cobranza, Supuestos!B80 = 60 (el VAN toma el capital de trabajo de la hoja Capital Trabajo y no depende de Ej_Flujo: no hace falta cambiar el desfase de la fila 6). Anotar VAN-TIR!C24 y restar el VAN base. Atención: con los datos actuales y este método, el VAN cambia ≈ ±USD 5,8M por ±5% de precio (≈ ±5,9M si el cambio se aplica a todo el año 1) y ≈ ∓USD 5,2M por ±5% de MP, muy por encima de lo que muestra la diapositiva de junio (±1,2M y ±1,0M); con un precio 5% menor, el VAN sería negativo (≈ −USD 3,0M). Tasa CP +2% y tipo de cambio ±10%: con este libro el VAN no cambia (el interés CP no entra al VAN y las proyecciones están en USD); informar ≈ 0 en VAN y, si se quiere mostrar, el efecto en la utilidad neta acumulada y en la caja (la tasa CP exige cambiar el 8% de cada fórmula de Ej_Flujo fila 17).</t>
         </is>
       </c>
       <c r="F89" s="367" t="inlineStr">
@@ -49930,6 +49930,7 @@
     <hyperlink ref="D80" location="'VAN-TIR'!C22" tooltip="Ir a 'VAN-TIR'!C22"/>
     <hyperlink ref="D85" location="'CONTROLES Y PPT'!B79" tooltip="Ir a 'CONTROLES Y PPT'!B79"/>
     <hyperlink ref="D86" location="'CONTROLES Y PPT'!B36" tooltip="Ir a 'CONTROLES Y PPT'!B36"/>
+    <hyperlink ref="D81" location="'PASO A PASO'!B92" tooltip="Ir al registro de actualizaciones"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToHeight="0"/>

</xml_diff>

<commit_message>
Guía de Alianza: ajustes de la verificación final (Word y Excel)
- Mapa del PPT: diap. 4 incluye el «61% inferior»; el peso de la MP pasa a las diap. 6, 11 y 13 (no a la 10).
- Roles en dividendos: la Gerencia presenta las alternativas y decide la Dirección.
- Excepción del rótulo Ej_Costos!P1 (paso D2), control de A1, notas de los indicadores 10, 22 y 33, total del anexo A y redacción de la sección 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4oZnCzWT5uwD7Y9gLbehx
</commit_message>
<xml_diff>
--- a/alianza/Informe_Financiero_ALIANZA_DEL_ACERO_INFORME2_09062026_AJUSTADO_A_10_AÑOS_CON_GUIA.xlsx
+++ b/alianza/Informe_Financiero_ALIANZA_DEL_ACERO_INFORME2_09062026_AJUSTADO_A_10_AÑOS_CON_GUIA.xlsx
@@ -45062,7 +45062,7 @@
       </c>
       <c r="H47" s="342" t="inlineStr">
         <is>
-          <t>Diap. 2 y 4 («39% del Plan»).</t>
+          <t>Diap. 2 y 4 («39% del Plan»; la diap. 4 dice además «61% inferior al Plan» = 1 − este valor).</t>
         </is>
       </c>
       <c r="I47" s="342"/>
@@ -45491,7 +45491,7 @@
       <c r="N58" s="342"/>
       <c r="O58" s="342"/>
     </row>
-    <row r="59" ht="17.2" customHeight="1">
+    <row r="59" ht="30.4" customHeight="1">
       <c r="B59" s="344">
         <v>22</v>
       </c>
@@ -45518,7 +45518,7 @@
       </c>
       <c r="H59" s="342" t="inlineStr">
         <is>
-          <t>Diap. 6. Plan en el libro: Ej_Costos!AE22/AE44 = 96,45% (el PPT dice 95,3%).</t>
+          <t>Diap. 6 (tabla «96.1%» y texto «&gt;96% de los costos variables»), 11 y 13 («&gt;96% de costos variables»). Plan en el libro: Ej_Costos!AE22/AE44 = 96,45% (el PPT dice 95,3%).</t>
         </is>
       </c>
       <c r="I59" s="342"/>
@@ -45936,7 +45936,7 @@
       </c>
       <c r="H70" s="342" t="inlineStr">
         <is>
-          <t>Diap. 8, 11 y 13 («USD 5-11,9M/año»). Hoy el año 7 es 4,0M.</t>
+          <t>Diap. 8 («USD 5-11.9M/año»), 11 y 13 («USD 5-12M/año»); el máximo también va en la diap. 2 («hasta USD 11.9M/año»). Hoy el año 7 es 4,0M.</t>
         </is>
       </c>
       <c r="I70" s="342"/>
@@ -48059,7 +48059,7 @@
       </c>
       <c r="C10" s="367" t="inlineStr">
         <is>
-          <t>Escribir solo en las celdas indicadas. No escribir en columnas de total o promedio (O y AD de Ej_Producción, Ej_Ingresos, Ej_Costos, Ej_Resultados y Ej_Deuda; O, AB, AO, BB, BO, CB, CO, DB, DO, EB y EF de Ej_Flujo), salvo las celdas que un paso indica expresamente: Ej_Producción!O31:O32 y O46:O47 (B4), Ej_Costos!O9:O19 y AD9:AD19 (B5), Ej_Costos!O1 (D2) y Ej_Flujo!O37 y O40 (E2). Tampoco en el plan original (columnas P y AE de esas cinco hojas; columna E de Supuestos). En Ej_Flujo no hay columnas de plan: P, AD y AE son meses (ene-2027, feb-2028 y mar-2028) y se editan cuando un paso lo indica. El auxiliar Ej_Costos!O88:P114 (paso D5) no es plan ni total.</t>
+          <t>Escribir solo en las celdas indicadas. No escribir en columnas de total o promedio (O y AD de Ej_Producción, Ej_Ingresos, Ej_Costos, Ej_Resultados y Ej_Deuda; O, AB, AO, BB, BO, CB, CO, DB, DO, EB y EF de Ej_Flujo), salvo las celdas que un paso indica expresamente: Ej_Producción!O31:O32 y O46:O47 (B4), Ej_Costos!O9:O19 y AD9:AD19 (B5), Ej_Costos!O1 (D2) y Ej_Flujo!O37 y O40 (E2). Tampoco en el plan original (columnas P y AE de esas cinco hojas, salvo el rótulo Ej_Costos!P1, que se actualiza en el paso D2; columna E de Supuestos). En Ej_Flujo no hay columnas de plan: P, AD y AE son meses (ene-2027, feb-2028 y mar-2028) y se editan cuando un paso lo indica. El auxiliar Ej_Costos!O88:P114 (paso D5) no es plan ni total.</t>
         </is>
       </c>
       <c r="D10" s="367"/>
@@ -48376,7 +48376,7 @@
       </c>
       <c r="F30" s="367" t="inlineStr">
         <is>
-          <t>Los nombres del libro y del PPT indican versión y fecha.</t>
+          <t>El nombre del libro indica versión y fecha (y, antes de empezar la fase G, también el del PPT).</t>
         </is>
       </c>
     </row>
@@ -49780,7 +49780,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="30.4" customHeight="1">
+    <row r="94" ht="43.6" customHeight="1">
       <c r="B94" s="369">
         <v>0</v>
       </c>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="E94" s="367" t="inlineStr">
         <is>
-          <t>Versión base usada en el PPT «Plan vs Actualizado 10 años» de junio 2026. Guía y controles agregados el 13/10/2026 sin modificar el modelo.</t>
+          <t>Versión base usada en el PPT «Plan vs Actualizado 10 años» de junio 2026. Guía y controles agregados el 13/10/2026 y actualizados el 16/10/2026, sin modificar el modelo.</t>
         </is>
       </c>
       <c r="F94" s="367" t="inlineStr">

</xml_diff>